<commit_message>
Add automatic duplicate transaction checks
</commit_message>
<xml_diff>
--- a/output/reconciliation_report.xlsx
+++ b/output/reconciliation_report.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Findings_by_type" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Exceptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Recon_bridge" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Outlier_review" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Matched_pairs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cleaning_log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings_by_type" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recon_bridge" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outlier_review" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched_pairs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning_log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings_by_type'!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Exceptions'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Recon_bridge'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Recon_bridge'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outlier_review'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Matched_pairs'!$A$1:$R$295</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cleaning_log'!$A$1:$D$2</definedName>
@@ -464,10 +464,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -595,8 +595,38 @@
         <v>0.07999999999999829</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>rows_with_null_keys</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>rows_with_invalid_values</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>rows_skipped_in_duplicate_check</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -788,22 +818,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Duplicates</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>POSSIBLE_DUPLICATE_INTERNAL</t>
+          <t>AMOUNT_MISMATCH</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>54.18</v>
+        <v>12.5</v>
       </c>
       <c r="F7" t="n">
-        <v>54.18</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="8">
@@ -814,22 +844,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>FX_MISMATCH</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>12.5</v>
+        <v>4.13</v>
       </c>
       <c r="F8" t="n">
-        <v>12.5</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="9">
@@ -840,22 +870,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FX</t>
+          <t>Fee</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FX_MISMATCH</t>
+          <t>NET_MISMATCH</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="F9" t="n">
-        <v>1.43</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="10">
@@ -871,43 +901,43 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NET_MISMATCH</t>
+          <t>FEE_ANOMALY</t>
         </is>
       </c>
       <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Duplicates</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>POSSIBLE_DUPLICATE_INTERNAL</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3.33</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Fee</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>FEE_ANOMALY</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
       <c r="E11" t="n">
-        <v>2.49</v>
+        <v>54.18</v>
       </c>
       <c r="F11" t="n">
-        <v>2.35</v>
+        <v>54.18</v>
       </c>
     </row>
     <row r="12">
@@ -1069,12 +1099,12 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>ledger REFUND -160.08 vs provider REFUND 160.03 (знак інвертовано); зсув балансу +320.11</t>
+          <t>ledger REFUND -160.08 vs provider REFUND 160.03 (sign inverted); balance shift +320.11</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Невідповідність типу/знаку (purchase↔refund): ефект на баланс = 2× суми.</t>
+          <t>Type/sign mismatch (purchase&lt;-&gt;refund): balance effect up to 2x the amount.</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1142,12 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>P00296 повторює P00041 (ідентичні суми та час); зайвий gross 217.15</t>
+          <t>P00296 repeats P00041 (identical amount and time); extra gross 217.15</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Один платіж розрахований двічі: ризик подвійного списання/виплати.</t>
+          <t>One payment settled twice: risk of double debit/payout.</t>
         </is>
       </c>
     </row>
@@ -1155,12 +1185,12 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>client_reference T202609-9999 відсутній у ledger; gross 146.8, fee 1.47</t>
+          <t>client_reference T202609-9999 is not in the ledger; gross 146.8, fee 1.47</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Провайдер розрахував операцію, якої немає в ledger: ризик фрод/збою обліку.</t>
+          <t>Provider settled a transaction that is not in the ledger: fraud or bookkeeping-failure risk.</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1228,12 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>ledger PURCHASE 21.42 vs provider REFUND 21.44; зсув балансу +0.02; якщо REFUND трактується як вихідний платіж — ризик до 2×21.42</t>
+          <t>ledger PURCHASE 21.42 vs provider REFUND 21.44; balance shift +0.02; if REFUND is treated as an outgoing payment, risk up to 2x21.42</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Невідповідність типу/знаку (purchase↔refund): ефект на баланс = 2× суми.</t>
+          <t>Type/sign mismatch (purchase&lt;-&gt;refund): balance effect up to 2x the amount.</t>
         </is>
       </c>
     </row>
@@ -1237,12 +1267,12 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>COMPLETED 2026-09-07 03:01; у provider-звіті (до 2026-09-13) немає, вік 155h</t>
+          <t>COMPLETED 2026-09-07 03:01; absent from the provider report (through 2026-09-13), age 155h</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>COMPLETED операція не розрахована провайдером: недоотримані кошти.</t>
+          <t>A COMPLETED transaction was not settled by the provider: funds not received.</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1310,12 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>internal status DECLINED, але settlement SETTLED gross 19.49</t>
+          <t>internal status DECLINED, but settlement SETTLED gross 19.49</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Відхилена операція пройшла settlement: гроші списано без валідної транзакції.</t>
+          <t>A declined transaction was settled: money moved without a valid transaction.</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1349,12 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>COMPLETED 2026-09-06 10:24; у provider-звіті (до 2026-09-13) немає, вік 172h</t>
+          <t>COMPLETED 2026-09-06 10:24; absent from the provider report (through 2026-09-13), age 172h</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>COMPLETED операція не розрахована провайдером: недоотримані кошти.</t>
+          <t>A COMPLETED transaction was not settled by the provider: funds not received.</t>
         </is>
       </c>
     </row>
@@ -1336,34 +1366,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Duplicates</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>POSSIBLE_DUPLICATE_INTERNAL</t>
+          <t>AMOUNT_MISMATCH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>T202609-0062</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>T202609-0077</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P00075</t>
+        </is>
+      </c>
       <c r="F9" t="n">
-        <v>54.18</v>
+        <v>12.5</v>
       </c>
       <c r="G9" t="n">
-        <v>54.18</v>
+        <v>12.5</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>T202609-0061 і T202609-0062: user U0042, merchant M017, 49.99 EUR, інтервал 2 хв; category 5732/7011, channel POS/IN_APP; обидві розраховані провайдером: так</t>
+          <t>ledger 2.19 vs provider 14.69 (Δ+12.50, tolerance ±0.25); gross is not derivable from original x provider_fx (=2.19) -&gt; amount error, not FX</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Схожі операції одного клієнта за хвилини: можливий double-charge.</t>
+          <t>Provider gross differs from ledger beyond the FX-noise tolerance.</t>
         </is>
       </c>
     </row>
@@ -1375,38 +1409,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Fee</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>NET_MISMATCH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T202609-0077</t>
+          <t>T202609-0275</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>P00075</t>
+          <t>P00253</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>12.5</v>
+        <v>3.33</v>
       </c>
       <c r="G10" t="n">
-        <v>12.5</v>
+        <v>3.33</v>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>ledger 2.19 vs provider 14.69 (Δ+12.50, допуск ±0.25); gross не виводиться з original×provider_fx (=2.19) → помилка суми, не FX</t>
+          <t>net 12.68 vs expected 9.35 (gross 9.52, fee 0.17)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Gross у провайдера ≠ ledger поза допуском FX-шуму.</t>
+          <t>net != gross -/+ fee: arithmetic error on the provider side.</t>
         </is>
       </c>
     </row>
@@ -1418,38 +1452,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fee</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NET_MISMATCH</t>
+          <t>FX_MISMATCH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>T202609-0275</t>
+          <t>T202609-0125</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>P00253</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3.33</v>
+        <v>2.78</v>
       </c>
       <c r="G11" t="n">
-        <v>3.33</v>
+        <v>2.78</v>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>net 12.68 vs очікуваний 9.35 (gross 9.52, fee 0.17)</t>
+          <t>USD: provider rate 1.0685 vs internal 0.9986 (+7.00%); provider +6.79% from currency median, internal -0.20% -&gt; provider is the deviating side</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>net ≠ gross ∓ fee: арифметична помилка у провайдера.</t>
+          <t>Provider FX rate deviates from the ledger and from the currency's normal range.</t>
         </is>
       </c>
     </row>
@@ -1461,38 +1495,38 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FX</t>
+          <t>Fee</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FX_MISMATCH</t>
+          <t>FEE_ANOMALY</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>T202609-0125</t>
+          <t>T202609-0188</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00172</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2.78</v>
+        <v>2.42</v>
       </c>
       <c r="G12" t="n">
-        <v>2.78</v>
+        <v>2.42</v>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>USD: provider rate 1.0685 vs internal 0.9986 (+7.00%); провайдер +6.79% від медіани валюти, internal -0.20% → відхиляється provider</t>
+          <t>fee 3.34 = 6.50% of 51.35; expected ≈0.92 (tiers ['1.8%', '1.0%'], min 0.05)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Курс провайдера відхиляється від ledger і від ринкового діапазону валюти.</t>
+          <t>Fee matches no known fee tier or minimum fee.</t>
         </is>
       </c>
     </row>
@@ -1504,38 +1538,38 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fee</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FEE_ANOMALY</t>
+          <t>FX_MISMATCH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>T202609-0188</t>
+          <t>T202609-0212</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>P00172</t>
+          <t>P00192</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.42</v>
+        <v>-1.35</v>
       </c>
       <c r="G13" t="n">
-        <v>2.42</v>
+        <v>1.35</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>fee 3.34 = 6.50% від 51.35; очікувалось ≈0.92 (тири ['1.8%', '1.0%'], мін 0.05)</t>
+          <t>USD: provider rate 0.9406 vs internal 1.0006 (-6.00%); provider -6.00% from currency median, internal +0.00% -&gt; provider is the deviating side</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Fee не відповідає жодному відомому тарифному тиру/мінімуму.</t>
+          <t>Provider FX rate deviates from the ledger and from the currency's normal range.</t>
         </is>
       </c>
     </row>
@@ -1547,81 +1581,77 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FX</t>
+          <t>Fee</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FX_MISMATCH</t>
+          <t>FEE_ANOMALY</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>T202609-0212</t>
+          <t>T202609-0248</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>P00192</t>
+          <t>P00226</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-1.35</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>1.35</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>USD: provider rate 0.9406 vs internal 1.0006 (-6.00%); провайдер -6.00% від медіани валюти, internal +0.00% → відхиляється provider</t>
+          <t>fee 0.01 = 0.12% of 8.44; expected ≈0.08 (tiers ['1.8%', '1.0%'], min 0.05)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Курс провайдера відхиляється від ledger і від ринкового діапазону валюти.</t>
+          <t>Fee matches no known fee tier or minimum fee.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fee</t>
+          <t>Duplicates</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FEE_ANOMALY</t>
+          <t>POSSIBLE_DUPLICATE_INTERNAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>T202609-0248</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>P00226</t>
-        </is>
-      </c>
+          <t>T202609-0062</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>-0.07000000000000001</v>
+        <v>54.18</v>
       </c>
       <c r="G15" t="n">
-        <v>0.07000000000000001</v>
+        <v>54.18</v>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>fee 0.01 = 0.12% від 8.44; очікувалось ≈0.08 (тири ['1.8%', '1.0%'], мін 0.05)</t>
+          <t>confidence LOW (channel, category differ): T202609-0061 and T202609-0062: user U0042, merchant M017, 49.99 EUR, gap 2 min; category 5732/7011, channel POS/IN_APP; both settled by provider: yes</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Fee не відповідає жодному відомому тарифному тиру/мінімуму.</t>
+          <t>Near-identical operations by one customer within minutes: possible double charge.</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1689,12 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>settlement через 268h (медіана 34h, p95 67h)</t>
+          <t>settled after 268h (median 34h, p95 67h)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Settlement значно пізніше за норму: cash-flow та ризик втрати запису.</t>
+          <t>Settlement far later than normal: cash-flow impact and risk of a lost record.</t>
         </is>
       </c>
     </row>
@@ -1698,12 +1728,12 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>8900.0 USD, robust z=5.5: суми, FX, fee, net, час — у нормі в обох джерелах; рекомендується лише бізнес-перевірка (ліміти, KYC/мерчант M020, категорія 5999)</t>
+          <t>8900.0 USD, robust z=5.5: amounts, FX, fee, net and timing are all normal in both sources; business review only (limits, KYC / merchant M020, category 5999)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Статистичний outlier, що звівся без розбіжностей: нормальна, але потребує business review.</t>
+          <t>Statistical outlier that reconciles cleanly: legitimate, but needs a business review.</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1761,74 +1791,94 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>+ Orphan settlements</t>
+          <t>− In flight (not yet due)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>146.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>+ Duplicate settlements</t>
+          <t>+ Orphan settlements</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>217.15</v>
+        <v>146.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>+ DECLINED settled</t>
+          <t>+ Duplicate settlements</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19.49</v>
+        <v>217.15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>± Sign/type mismatch</t>
+          <t>+ DECLINED settled</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>320.13</v>
+        <v>19.49</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>± Amount/FX mismatch</t>
+          <t>± Sign/type mismatch</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13.93</v>
+        <v>320.13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>± Нормальний FX-шум (решта)</t>
+          <t>± Amount/FX mismatch</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>13.93</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>± Rows with null amounts (not comparable)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>± Normal FX noise (remainder)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>-4.23</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10">
-        <f> Provider gross (всі рядки)</f>
+    <row r="12">
+      <c r="A12">
+        <f> Provider gross (all rows)</f>
         <v/>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" t="n">
         <v>17886.83</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>